<commit_message>
feat: read products from excel
</commit_message>
<xml_diff>
--- a/data/ma-products.xlsx
+++ b/data/ma-products.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/55cf92656b64c0cb/Документи/Market-Intelligence-Agent/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{AF41C6E9-2D12-4B59-9C0C-221F2C13FEE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6203F639-940C-4F53-B46D-61ABC44C4F5C}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="8_{AF41C6E9-2D12-4B59-9C0C-221F2C13FEE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85B41058-F7C9-4629-B409-8D299EA0C2B2}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EC267631-31B5-4518-9F5C-42AAE75C3943}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{EC267631-31B5-4518-9F5C-42AAE75C3943}"/>
   </bookViews>
   <sheets>
-    <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
+    <sheet name="MA-Produkte" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,9 +47,6 @@
     <t>EAN</t>
   </si>
   <si>
-    <t>MPN / Hersteller-Nr.</t>
-  </si>
-  <si>
     <t>Produktname</t>
   </si>
   <si>
@@ -59,12 +56,6 @@
     <t>Kategorie</t>
   </si>
   <si>
-    <t>MA-Preis</t>
-  </si>
-  <si>
-    <t>MA-Link</t>
-  </si>
-  <si>
     <t>MA-10001</t>
   </si>
   <si>
@@ -135,6 +126,15 @@
   </si>
   <si>
     <t>https://www.ma-versand.de/ersatzteile/fuer-motoren/...</t>
+  </si>
+  <si>
+    <t>MPN</t>
+  </si>
+  <si>
+    <t>MA Preis</t>
+  </si>
+  <si>
+    <t>MA Link</t>
   </si>
 </sst>
 </file>
@@ -142,7 +142,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="#,##0.00\ [$€-1];[Red]\-#,##0.00\ [$€-1]"/>
+    <numFmt numFmtId="164" formatCode="#,##0.00\ [$€-1];[Red]\-#,##0.00\ [$€-1]"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -201,7 +201,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
@@ -223,6 +223,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -552,7 +556,7 @@
     <col min="8" max="8" width="56.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -560,152 +564,152 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>9</v>
       </c>
       <c r="C2" s="3">
         <v>532406713</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G2" s="4">
         <v>24.99</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>18</v>
       </c>
       <c r="G3" s="4">
         <v>6.9</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C4" s="3">
         <v>532187256</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G4" s="4">
         <v>39.9</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>26</v>
       </c>
       <c r="G5" s="4">
         <v>12.9</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>30</v>
       </c>
       <c r="G6" s="4">
         <v>25.9</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>